<commit_message>
updated 31/3-maybe missed one inv
</commit_message>
<xml_diff>
--- a/src/DayBook_all.xlsx
+++ b/src/DayBook_all.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J2373"/>
+  <dimension ref="A1:J2374"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="10" max="10" width="20.7109375" style="2" customWidth="1"/>
@@ -87907,7 +87907,7 @@
     <row r="2314">
       <c r="A2314" t="inlineStr">
         <is>
-          <t>A ONE STEELS INDIA LIMITED-GBD</t>
+          <t>A One Ispat Private Ltd</t>
         </is>
       </c>
       <c r="B2314" t="inlineStr">
@@ -87916,22 +87916,22 @@
         </is>
       </c>
       <c r="C2314">
-        <v>2285386.5</v>
+        <v>2470014</v>
       </c>
       <c r="D2314">
-        <v>411369.57</v>
+        <v>444602.52</v>
       </c>
       <c r="E2314">
-        <v>2696756</v>
+        <v>2914617.56</v>
       </c>
       <c r="F2314">
-        <v>287.47</v>
+        <v>312.66</v>
       </c>
       <c r="G2314">
-        <v>7950.000000000001</v>
+        <v>7900</v>
       </c>
       <c r="H2314">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I2314" t="inlineStr">
         <is>
@@ -87945,7 +87945,7 @@
     <row r="2315">
       <c r="A2315" t="inlineStr">
         <is>
-          <t>A One Ispat Private Ltd</t>
+          <t>A ONE STEELS INDIA LIMITED-GBD</t>
         </is>
       </c>
       <c r="B2315" t="inlineStr">
@@ -87954,22 +87954,22 @@
         </is>
       </c>
       <c r="C2315">
-        <v>2189722</v>
+        <v>2285386.5</v>
       </c>
       <c r="D2315">
-        <v>394149.96</v>
+        <v>411369.57</v>
       </c>
       <c r="E2315">
-        <v>2583873</v>
+        <v>2696756</v>
       </c>
       <c r="F2315">
-        <v>277.18</v>
+        <v>287.47</v>
       </c>
       <c r="G2315">
-        <v>7900</v>
+        <v>7950.000000000001</v>
       </c>
       <c r="H2315">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I2315" t="inlineStr">
         <is>
@@ -88021,7 +88021,7 @@
     <row r="2317">
       <c r="A2317" t="inlineStr">
         <is>
-          <t>M S METALS &amp; STEELS PRIVATE LIMITED - TN - Unit 1</t>
+          <t>KUBAIR STEEL AND POWER LLP</t>
         </is>
       </c>
       <c r="B2317" t="inlineStr">
@@ -88030,26 +88030,26 @@
         </is>
       </c>
       <c r="C2317">
-        <v>1487910.5</v>
+        <v>1310180</v>
       </c>
       <c r="D2317">
-        <v>267823.89</v>
+        <v>235832.4</v>
       </c>
       <c r="E2317">
-        <v>1755733</v>
+        <v>1546012.6</v>
       </c>
       <c r="F2317">
-        <v>164.41</v>
+        <v>166.82</v>
       </c>
       <c r="G2317">
-        <v>9050</v>
+        <v>7853.85445390241</v>
       </c>
       <c r="H2317">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I2317" t="inlineStr">
         <is>
-          <t>Abhijit Maloo</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="J2317" s="2">
@@ -88059,7 +88059,7 @@
     <row r="2318">
       <c r="A2318" t="inlineStr">
         <is>
-          <t>Sugna Sponge &amp; Power Pvt Ltd</t>
+          <t>M S METALS &amp; STEELS PRIVATE LIMITED - TN - Unit 1</t>
         </is>
       </c>
       <c r="B2318" t="inlineStr">
@@ -88068,26 +88068,26 @@
         </is>
       </c>
       <c r="C2318">
-        <v>1269138</v>
+        <v>1487910.5</v>
       </c>
       <c r="D2318">
-        <v>258939.36</v>
+        <v>267823.89</v>
       </c>
       <c r="E2318">
-        <v>1619517.36</v>
+        <v>1755733</v>
       </c>
       <c r="F2318">
-        <v>162.71</v>
+        <v>164.41</v>
       </c>
       <c r="G2318">
-        <v>7800.000000000001</v>
+        <v>9050</v>
       </c>
       <c r="H2318">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I2318" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Abhijit Maloo</t>
         </is>
       </c>
       <c r="J2318" s="2">
@@ -88097,7 +88097,7 @@
     <row r="2319">
       <c r="A2319" t="inlineStr">
         <is>
-          <t>KUBAIR STEEL AND POWER LLP</t>
+          <t>Sugna Sponge &amp; Power Pvt Ltd</t>
         </is>
       </c>
       <c r="B2319" t="inlineStr">
@@ -88106,22 +88106,22 @@
         </is>
       </c>
       <c r="C2319">
-        <v>1292160</v>
+        <v>1269138</v>
       </c>
       <c r="D2319">
-        <v>232588.8</v>
+        <v>258939.36</v>
       </c>
       <c r="E2319">
-        <v>1524749</v>
+        <v>1619517.36</v>
       </c>
       <c r="F2319">
-        <v>161.52</v>
+        <v>162.71</v>
       </c>
       <c r="G2319">
-        <v>7999.999999999999</v>
+        <v>7800.000000000001</v>
       </c>
       <c r="H2319">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I2319" t="inlineStr">
         <is>
@@ -89873,7 +89873,7 @@
       </c>
       <c r="I2365" t="inlineStr">
         <is>
-          <t>Shresth Maheshwari</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="J2365" s="2">
@@ -89883,35 +89883,35 @@
     <row r="2366">
       <c r="A2366" t="inlineStr">
         <is>
-          <t>Pulkit Metals Pvt Ltd</t>
+          <t>Jai Hind Rolling Mills India Pvt Limited</t>
         </is>
       </c>
       <c r="B2366" t="inlineStr">
         <is>
-          <t>Tundish Ramming Mix</t>
+          <t>Nali Top</t>
         </is>
       </c>
       <c r="C2366">
-        <v>135000</v>
+        <v>19754</v>
       </c>
       <c r="D2366">
-        <v>24300</v>
+        <v>3555.72</v>
       </c>
       <c r="E2366">
-        <v>159300</v>
+        <v>23309.72</v>
       </c>
       <c r="F2366">
-        <v>5</v>
+        <v>5.81</v>
       </c>
       <c r="G2366">
-        <v>27000</v>
+        <v>3400</v>
       </c>
       <c r="H2366">
         <v>1</v>
       </c>
       <c r="I2366" t="inlineStr">
         <is>
-          <t>Abhijit Maloo</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="J2366" s="2">
@@ -89921,35 +89921,35 @@
     <row r="2367">
       <c r="A2367" t="inlineStr">
         <is>
-          <t>ADRI STEEL PRIVATE LIMITED</t>
+          <t>Pulkit Metals Pvt Ltd</t>
         </is>
       </c>
       <c r="B2367" t="inlineStr">
         <is>
-          <t>Nali Top</t>
+          <t>Tundish Ramming Mix</t>
         </is>
       </c>
       <c r="C2367">
-        <v>15744</v>
+        <v>135000</v>
       </c>
       <c r="D2367">
-        <v>0</v>
+        <v>24300</v>
       </c>
       <c r="E2367">
-        <v>18577.92</v>
+        <v>159300</v>
       </c>
       <c r="F2367">
-        <v>4.92</v>
+        <v>5</v>
       </c>
       <c r="G2367">
-        <v>3200</v>
+        <v>27000</v>
       </c>
       <c r="H2367">
         <v>1</v>
       </c>
       <c r="I2367" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Abhijit Maloo</t>
         </is>
       </c>
       <c r="J2367" s="2">
@@ -89959,26 +89959,31 @@
     <row r="2368">
       <c r="A2368" t="inlineStr">
         <is>
-          <t>Mahrishi Meltchems Pvt Ltd</t>
+          <t>ADRI STEEL PRIVATE LIMITED</t>
+        </is>
+      </c>
+      <c r="B2368" t="inlineStr">
+        <is>
+          <t>Nali Top</t>
         </is>
       </c>
       <c r="C2368">
-        <v>556000</v>
+        <v>15744</v>
       </c>
       <c r="D2368">
-        <v>100080</v>
+        <v>0</v>
       </c>
       <c r="E2368">
-        <v>656080</v>
+        <v>18577.92</v>
       </c>
       <c r="F2368">
-        <v>4</v>
+        <v>4.92</v>
       </c>
       <c r="G2368">
-        <v>139000</v>
+        <v>3200</v>
       </c>
       <c r="H2368">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I2368" t="inlineStr">
         <is>
@@ -89996,22 +90001,22 @@
         </is>
       </c>
       <c r="C2369">
-        <v>1145500</v>
+        <v>556000</v>
       </c>
       <c r="D2369">
-        <v>206190</v>
+        <v>100080</v>
       </c>
       <c r="E2369">
-        <v>1351690</v>
+        <v>656080</v>
       </c>
       <c r="F2369">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="G2369">
-        <v>327285.7142857143</v>
+        <v>139000</v>
       </c>
       <c r="H2369">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I2369" t="inlineStr">
         <is>
@@ -90025,31 +90030,26 @@
     <row r="2370">
       <c r="A2370" t="inlineStr">
         <is>
-          <t>SNAM ALLOYS PRIVATE LIMITED</t>
-        </is>
-      </c>
-      <c r="B2370" t="inlineStr">
-        <is>
-          <t>Ordinary Ramming Mass</t>
+          <t>Mahrishi Meltchems Pvt Ltd</t>
         </is>
       </c>
       <c r="C2370">
-        <v>11836</v>
+        <v>1145500</v>
       </c>
       <c r="D2370">
-        <v>29098.08</v>
+        <v>206190</v>
       </c>
       <c r="E2370">
-        <v>13966.48</v>
+        <v>1351690</v>
       </c>
       <c r="F2370">
-        <v>2.69</v>
+        <v>3.5</v>
       </c>
       <c r="G2370">
-        <v>4400</v>
+        <v>327285.7142857143</v>
       </c>
       <c r="H2370">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I2370" t="inlineStr">
         <is>
@@ -90063,28 +90063,28 @@
     <row r="2371">
       <c r="A2371" t="inlineStr">
         <is>
-          <t>SRI BHAVANI CASTINGS LTD</t>
+          <t>SNAM ALLOYS PRIVATE LIMITED</t>
         </is>
       </c>
       <c r="B2371" t="inlineStr">
         <is>
-          <t>Boric Acid Premix</t>
+          <t>Ordinary Ramming Mass</t>
         </is>
       </c>
       <c r="C2371">
-        <v>9200</v>
+        <v>11836</v>
       </c>
       <c r="D2371">
-        <v>0</v>
+        <v>29098.08</v>
       </c>
       <c r="E2371">
-        <v>10856</v>
+        <v>13966.48</v>
       </c>
       <c r="F2371">
-        <v>1</v>
+        <v>2.69</v>
       </c>
       <c r="G2371">
-        <v>9200</v>
+        <v>4400</v>
       </c>
       <c r="H2371">
         <v>1</v>
@@ -90106,23 +90106,23 @@
       </c>
       <c r="B2372" t="inlineStr">
         <is>
-          <t>Boron Oxide Premix</t>
+          <t>Boric Acid Premix</t>
         </is>
       </c>
       <c r="C2372">
-        <v>10800</v>
+        <v>9200</v>
       </c>
       <c r="D2372">
-        <v>3600</v>
+        <v>0</v>
       </c>
       <c r="E2372">
-        <v>12744</v>
+        <v>10856</v>
       </c>
       <c r="F2372">
         <v>1</v>
       </c>
       <c r="G2372">
-        <v>10800</v>
+        <v>9200</v>
       </c>
       <c r="H2372">
         <v>1</v>
@@ -90139,23 +90139,28 @@
     <row r="2373">
       <c r="A2373" t="inlineStr">
         <is>
-          <t>RDTMT Steels India Pvt Ltd</t>
+          <t>SRI BHAVANI CASTINGS LTD</t>
+        </is>
+      </c>
+      <c r="B2373" t="inlineStr">
+        <is>
+          <t>Boron Oxide Premix</t>
         </is>
       </c>
       <c r="C2373">
-        <v>8500</v>
+        <v>10800</v>
       </c>
       <c r="D2373">
-        <v>1530</v>
+        <v>3600</v>
       </c>
       <c r="E2373">
-        <v>10030</v>
+        <v>12744</v>
       </c>
       <c r="F2373">
-        <v>0.05</v>
+        <v>1</v>
       </c>
       <c r="G2373">
-        <v>170000</v>
+        <v>10800</v>
       </c>
       <c r="H2373">
         <v>1</v>
@@ -90166,6 +90171,39 @@
         </is>
       </c>
       <c r="J2373" s="2">
+        <v>46082</v>
+      </c>
+    </row>
+    <row r="2374">
+      <c r="A2374" t="inlineStr">
+        <is>
+          <t>RDTMT Steels India Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="C2374">
+        <v>8500</v>
+      </c>
+      <c r="D2374">
+        <v>1530</v>
+      </c>
+      <c r="E2374">
+        <v>10030</v>
+      </c>
+      <c r="F2374">
+        <v>0.05</v>
+      </c>
+      <c r="G2374">
+        <v>170000</v>
+      </c>
+      <c r="H2374">
+        <v>1</v>
+      </c>
+      <c r="I2374" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J2374" s="2">
         <v>46082</v>
       </c>
     </row>

</xml_diff>